<commit_message>
simulate from elo and proba
</commit_message>
<xml_diff>
--- a/runapp/www/round32assignment.xlsx
+++ b/runapp/www/round32assignment.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\loicl\OneDrive\Documents\Loïc\Divers_non_disque\Data_science\Projet\MesProjets\Coupe_du_monde_2026\runapp\www\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4E820F97-DECF-4E6F-BA44-7FBB93C66C1E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F610A1CD-58B5-493A-94E5-7F9B315A0985}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-21060" yWindow="-1110" windowWidth="17280" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="132" uniqueCount="64">
   <si>
     <t>id</t>
   </si>
@@ -85,6 +85,138 @@
   </si>
   <si>
     <t>id_2</t>
+  </si>
+  <si>
+    <t>Match</t>
+  </si>
+  <si>
+    <t>Round of 32 1</t>
+  </si>
+  <si>
+    <t>Round of 32 2</t>
+  </si>
+  <si>
+    <t>Round of 32 3</t>
+  </si>
+  <si>
+    <t>Round of 32 4</t>
+  </si>
+  <si>
+    <t>Round of 32 5</t>
+  </si>
+  <si>
+    <t>Round of 32 6</t>
+  </si>
+  <si>
+    <t>Round of 32 7</t>
+  </si>
+  <si>
+    <t>Round of 32 8</t>
+  </si>
+  <si>
+    <t>Round of 32 9</t>
+  </si>
+  <si>
+    <t>Round of 32 10</t>
+  </si>
+  <si>
+    <t>Round of 32 11</t>
+  </si>
+  <si>
+    <t>Round of 32 12</t>
+  </si>
+  <si>
+    <t>Round of 32 13</t>
+  </si>
+  <si>
+    <t>Round of 32 14</t>
+  </si>
+  <si>
+    <t>Round of 32 15</t>
+  </si>
+  <si>
+    <t>Round of 32 16</t>
+  </si>
+  <si>
+    <t>round of 16 1</t>
+  </si>
+  <si>
+    <t>round of 16 2</t>
+  </si>
+  <si>
+    <t>round of 16 3</t>
+  </si>
+  <si>
+    <t>round of 16 4</t>
+  </si>
+  <si>
+    <t>round of 16 5</t>
+  </si>
+  <si>
+    <t>round of 16 6</t>
+  </si>
+  <si>
+    <t>round of 16 7</t>
+  </si>
+  <si>
+    <t>round of 16 8</t>
+  </si>
+  <si>
+    <t>Quarter 1</t>
+  </si>
+  <si>
+    <t>Quarter 2</t>
+  </si>
+  <si>
+    <t>Quarter 3</t>
+  </si>
+  <si>
+    <t>Quarter 4</t>
+  </si>
+  <si>
+    <t>Semi 1</t>
+  </si>
+  <si>
+    <t>Semi 2</t>
+  </si>
+  <si>
+    <t>Finale</t>
+  </si>
+  <si>
+    <t>Third_match</t>
+  </si>
+  <si>
+    <t>Winner</t>
+  </si>
+  <si>
+    <t>Round of 16</t>
+  </si>
+  <si>
+    <t>Match_type</t>
+  </si>
+  <si>
+    <t>Round of 32</t>
+  </si>
+  <si>
+    <t>Quarter</t>
+  </si>
+  <si>
+    <t>Semi</t>
+  </si>
+  <si>
+    <t>Final</t>
+  </si>
+  <si>
+    <t>Third place</t>
+  </si>
+  <si>
+    <t>Loser</t>
+  </si>
+  <si>
+    <t>Next_opponent</t>
+  </si>
+  <si>
+    <t>ID</t>
   </si>
 </sst>
 </file>
@@ -420,44 +552,65 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H18"/>
+  <dimension ref="A1:N33"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="12.109375" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="13.33203125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="7.33203125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.109375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="13.33203125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="7.33203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="13.77734375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="13.33203125" customWidth="1"/>
+    <col min="6" max="6" width="12.109375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="13.33203125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="7.33203125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="12.109375" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="13.33203125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="7.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>1</v>
+        <v>63</v>
       </c>
       <c r="C1" t="s">
-        <v>2</v>
+        <v>20</v>
       </c>
       <c r="D1" t="s">
+        <v>62</v>
+      </c>
+      <c r="E1" t="s">
+        <v>55</v>
+      </c>
+      <c r="F1" t="s">
+        <v>1</v>
+      </c>
+      <c r="G1" t="s">
+        <v>2</v>
+      </c>
+      <c r="H1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="I1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="J1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="K1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="L1" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="M1" t="s">
+        <v>53</v>
+      </c>
+      <c r="N1" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="2" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A2" s="1">
         <v>74</v>
       </c>
@@ -465,342 +618,752 @@
         <v>1</v>
       </c>
       <c r="C2" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="F2" s="1">
+        <v>1</v>
+      </c>
+      <c r="G2" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="D2" s="2"/>
-      <c r="E2" s="1">
+      <c r="H2" s="2"/>
+      <c r="I2" s="1">
         <v>3</v>
       </c>
-      <c r="F2" s="1"/>
-      <c r="G2" s="2"/>
-      <c r="H2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="J2" s="1"/>
+      <c r="K2" s="2"/>
+      <c r="L2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A3" s="1">
         <v>77</v>
       </c>
       <c r="B3" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C3" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="E3" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="F3" s="1">
+        <v>1</v>
+      </c>
+      <c r="G3" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="D3" s="2"/>
-      <c r="E3" s="1">
+      <c r="H3" s="2"/>
+      <c r="I3" s="1">
         <v>3</v>
       </c>
-      <c r="F3" s="1"/>
-      <c r="G3" s="2"/>
-      <c r="H3">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="J3" s="1"/>
+      <c r="K3" s="2"/>
+      <c r="L3">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="4" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A4" s="1">
         <v>73</v>
       </c>
       <c r="B4" s="1">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C4" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="E4" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="F4" s="1">
+        <v>2</v>
+      </c>
+      <c r="G4" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="D4" s="2"/>
-      <c r="E4" s="1">
-        <v>2</v>
-      </c>
-      <c r="F4" s="1" t="s">
+      <c r="H4" s="2"/>
+      <c r="I4" s="1">
+        <v>2</v>
+      </c>
+      <c r="J4" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="G4" s="2"/>
-      <c r="H4">
+      <c r="K4" s="2"/>
+      <c r="L4">
         <v>3</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A5" s="1">
         <v>75</v>
       </c>
       <c r="B5" s="1">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C5" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="E5" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="F5" s="1">
+        <v>1</v>
+      </c>
+      <c r="G5" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="D5" s="2"/>
-      <c r="E5" s="1">
-        <v>2</v>
-      </c>
-      <c r="F5" s="1" t="s">
+      <c r="H5" s="2"/>
+      <c r="I5" s="1">
+        <v>2</v>
+      </c>
+      <c r="J5" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="G5" s="2"/>
-      <c r="H5">
+      <c r="K5" s="2"/>
+      <c r="L5">
         <v>4</v>
       </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A6" s="1">
         <v>83</v>
       </c>
       <c r="B6" s="1">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="C6" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="E6" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="F6" s="1">
+        <v>2</v>
+      </c>
+      <c r="G6" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="D6" s="2"/>
-      <c r="E6" s="1">
-        <v>2</v>
-      </c>
-      <c r="F6" s="1" t="s">
+      <c r="H6" s="2"/>
+      <c r="I6" s="1">
+        <v>2</v>
+      </c>
+      <c r="J6" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="G6" s="2"/>
-      <c r="H6">
+      <c r="K6" s="2"/>
+      <c r="L6">
         <v>5</v>
       </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A7" s="1">
         <v>84</v>
       </c>
       <c r="B7" s="1">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="C7" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="D7" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="E7" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="F7" s="1">
+        <v>1</v>
+      </c>
+      <c r="G7" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="D7" s="2"/>
-      <c r="E7" s="1">
-        <v>2</v>
-      </c>
-      <c r="F7" s="1" t="s">
+      <c r="H7" s="2"/>
+      <c r="I7" s="1">
+        <v>2</v>
+      </c>
+      <c r="J7" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="G7" s="2"/>
-      <c r="H7">
+      <c r="K7" s="2"/>
+      <c r="L7">
         <v>6</v>
       </c>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A8" s="1">
         <v>81</v>
       </c>
       <c r="B8" s="1">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="C8" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="D8" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="E8" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="F8" s="1">
+        <v>1</v>
+      </c>
+      <c r="G8" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="D8" s="2"/>
-      <c r="E8" s="1">
+      <c r="H8" s="2"/>
+      <c r="I8" s="1">
         <v>3</v>
       </c>
-      <c r="F8" s="1"/>
-      <c r="G8" s="2"/>
-      <c r="H8">
+      <c r="J8" s="1"/>
+      <c r="K8" s="2"/>
+      <c r="L8">
         <v>7</v>
       </c>
     </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A9" s="1">
         <v>82</v>
       </c>
       <c r="B9" s="1">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="C9" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="D9" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="E9" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="F9" s="1">
+        <v>1</v>
+      </c>
+      <c r="G9" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="D9" s="2"/>
-      <c r="E9" s="1">
+      <c r="H9" s="2"/>
+      <c r="I9" s="1">
         <v>3</v>
       </c>
-      <c r="F9" s="1"/>
-      <c r="G9" s="2"/>
-      <c r="H9">
+      <c r="J9" s="1"/>
+      <c r="K9" s="2"/>
+      <c r="L9">
         <v>8</v>
       </c>
     </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A10" s="1">
         <v>76</v>
       </c>
       <c r="B10" s="1">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="C10" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="D10" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="E10" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="F10" s="1">
+        <v>1</v>
+      </c>
+      <c r="G10" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="D10" s="2"/>
-      <c r="E10" s="1">
-        <v>2</v>
-      </c>
-      <c r="F10" s="1" t="s">
+      <c r="H10" s="2"/>
+      <c r="I10" s="1">
+        <v>2</v>
+      </c>
+      <c r="J10" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="G10" s="2"/>
-      <c r="H10">
+      <c r="K10" s="2"/>
+      <c r="L10">
         <v>9</v>
       </c>
     </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A11" s="1">
         <v>78</v>
       </c>
       <c r="B11" s="1">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="C11" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="D11" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="E11" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="F11" s="1">
+        <v>2</v>
+      </c>
+      <c r="G11" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="D11" s="2"/>
-      <c r="E11" s="1">
-        <v>2</v>
-      </c>
-      <c r="F11" s="1" t="s">
+      <c r="H11" s="2"/>
+      <c r="I11" s="1">
+        <v>2</v>
+      </c>
+      <c r="J11" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="G11" s="2"/>
-      <c r="H11">
+      <c r="K11" s="2"/>
+      <c r="L11">
         <v>10</v>
       </c>
     </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A12" s="1">
         <v>79</v>
       </c>
       <c r="B12" s="1">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="C12" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="D12" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="E12" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="F12" s="1">
+        <v>1</v>
+      </c>
+      <c r="G12" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="D12" s="2"/>
-      <c r="E12" s="1">
+      <c r="H12" s="2"/>
+      <c r="I12" s="1">
         <v>3</v>
       </c>
-      <c r="F12" s="1"/>
-      <c r="G12" s="2"/>
-      <c r="H12">
+      <c r="J12" s="1"/>
+      <c r="K12" s="2"/>
+      <c r="L12">
         <v>11</v>
       </c>
     </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A13" s="1">
         <v>80</v>
       </c>
       <c r="B13" s="1">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="C13" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="D13" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="E13" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="F13" s="1">
+        <v>1</v>
+      </c>
+      <c r="G13" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="D13" s="2"/>
-      <c r="E13" s="1">
+      <c r="H13" s="2"/>
+      <c r="I13" s="1">
         <v>3</v>
       </c>
-      <c r="F13" s="1"/>
-      <c r="G13" s="2"/>
-      <c r="H13">
+      <c r="J13" s="1"/>
+      <c r="K13" s="2"/>
+      <c r="L13">
         <v>12</v>
       </c>
     </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A14" s="1">
         <v>86</v>
       </c>
       <c r="B14" s="1">
-        <v>1</v>
+        <v>13</v>
       </c>
       <c r="C14" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="D14" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="E14" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="F14" s="1">
+        <v>1</v>
+      </c>
+      <c r="G14" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="D14" s="2"/>
-      <c r="E14" s="1">
-        <v>2</v>
-      </c>
-      <c r="F14" s="1" t="s">
+      <c r="H14" s="2"/>
+      <c r="I14" s="1">
+        <v>2</v>
+      </c>
+      <c r="J14" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="G14" s="2"/>
-      <c r="H14">
+      <c r="K14" s="2"/>
+      <c r="L14">
         <v>13</v>
       </c>
     </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A15" s="1">
         <v>88</v>
       </c>
       <c r="B15" s="1">
-        <v>2</v>
+        <v>14</v>
       </c>
       <c r="C15" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="D15" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="E15" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="F15" s="1">
+        <v>2</v>
+      </c>
+      <c r="G15" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="D15" s="2"/>
-      <c r="E15" s="1">
-        <v>2</v>
-      </c>
-      <c r="F15" s="1" t="s">
+      <c r="H15" s="2"/>
+      <c r="I15" s="1">
+        <v>2</v>
+      </c>
+      <c r="J15" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="G15" s="2"/>
-      <c r="H15">
+      <c r="K15" s="2"/>
+      <c r="L15">
         <v>14</v>
       </c>
     </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A16" s="1">
         <v>85</v>
       </c>
       <c r="B16" s="1">
-        <v>1</v>
+        <v>15</v>
       </c>
       <c r="C16" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="D16" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="E16" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="F16" s="1">
+        <v>1</v>
+      </c>
+      <c r="G16" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="D16" s="2"/>
-      <c r="E16" s="1">
+      <c r="H16" s="2"/>
+      <c r="I16" s="1">
         <v>3</v>
       </c>
-      <c r="F16" s="1"/>
-      <c r="G16" s="2"/>
-      <c r="H16">
+      <c r="J16" s="1"/>
+      <c r="K16" s="2"/>
+      <c r="L16">
         <v>15</v>
       </c>
     </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A17" s="1">
         <v>87</v>
       </c>
       <c r="B17" s="1">
-        <v>1</v>
+        <v>16</v>
       </c>
       <c r="C17" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="D17" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="E17" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="F17" s="1">
+        <v>1</v>
+      </c>
+      <c r="G17" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="D17" s="2"/>
-      <c r="E17" s="1">
+      <c r="H17" s="2"/>
+      <c r="I17" s="1">
         <v>3</v>
       </c>
-      <c r="F17" s="1"/>
-      <c r="G17" s="2"/>
-      <c r="H17">
+      <c r="J17" s="1"/>
+      <c r="K17" s="2"/>
+      <c r="L17">
         <v>16</v>
       </c>
     </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A18" s="1"/>
-      <c r="B18" s="1"/>
-      <c r="C18" s="1"/>
-      <c r="D18" s="1"/>
-      <c r="E18" s="1"/>
+      <c r="B18" s="1">
+        <v>17</v>
+      </c>
+      <c r="C18" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="D18" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="E18" s="1" t="s">
+        <v>54</v>
+      </c>
       <c r="F18" s="1"/>
       <c r="G18" s="1"/>
+      <c r="H18" s="1"/>
+      <c r="I18" s="1"/>
+      <c r="J18" s="1"/>
+      <c r="K18" s="1"/>
+    </row>
+    <row r="19" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="B19" s="1">
+        <v>18</v>
+      </c>
+      <c r="C19" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="D19" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="E19" s="1" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="20" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="B20" s="1">
+        <v>19</v>
+      </c>
+      <c r="C20" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="D20" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="E20" s="1" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="21" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="B21" s="1">
+        <v>20</v>
+      </c>
+      <c r="C21" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="D21" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="E21" s="1" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="22" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="B22" s="1">
+        <v>21</v>
+      </c>
+      <c r="C22" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="D22" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="E22" s="1" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="23" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="B23" s="1">
+        <v>22</v>
+      </c>
+      <c r="C23" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="D23" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="E23" s="1" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="24" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="B24" s="1">
+        <v>23</v>
+      </c>
+      <c r="C24" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="D24" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="E24" s="1" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="25" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="B25" s="1">
+        <v>24</v>
+      </c>
+      <c r="C25" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="D25" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="E25" s="1" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="26" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="B26" s="1">
+        <v>25</v>
+      </c>
+      <c r="C26" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="D26" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="E26" s="1" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="27" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="B27" s="1">
+        <v>26</v>
+      </c>
+      <c r="C27" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="D27" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="E27" s="1" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="28" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="B28" s="1">
+        <v>27</v>
+      </c>
+      <c r="C28" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="D28" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="E28" s="1" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="29" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="B29" s="1">
+        <v>28</v>
+      </c>
+      <c r="C29" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="D29" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="E29" s="1" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="30" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="B30" s="1">
+        <v>29</v>
+      </c>
+      <c r="C30" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="D30" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="E30" s="1" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="31" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="B31" s="1">
+        <v>30</v>
+      </c>
+      <c r="C31" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="D31" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="E31" s="1" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="32" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="B32" s="1">
+        <v>31</v>
+      </c>
+      <c r="C32" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="D32" s="1"/>
+      <c r="E32" s="1" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="33" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="B33" s="1">
+        <v>32</v>
+      </c>
+      <c r="C33" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="D33" s="1"/>
+      <c r="E33" s="1" t="s">
+        <v>60</v>
+      </c>
     </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>

</xml_diff>